<commit_message>
Make article 4 of the fund decree explicit in criteria documents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHwNN6RfVzTYVCS9bRLUAz
</commit_message>
<xml_diff>
--- a/entregables/Herramienta_priorizacion_FEAC_BCS.xlsx
+++ b/entregables/Herramienta_priorizacion_FEAC_BCS.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="435">
   <si>
     <t xml:space="preserve">Herramienta de elegibilidad y priorización de proyectos – FEAC BCS</t>
   </si>
@@ -35,13 +35,19 @@
     <t xml:space="preserve">Fondo Estatal Ambiental y Climático de Baja California Sur · aplica el documento «Criterios de elegibilidad y selección de proyectos – FEAC BCS».</t>
   </si>
   <si>
+    <t xml:space="preserve">Qué es el artículo 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El artículo 4 del Decreto por el que se constituye el Fideicomiso Público denominado Fondo Estatal Ambiental y Climático de Baja California Sur establece los fines del Fondo: 16 fracciones (I a XVI) que definen en qué puede invertir sus recursos. En esta herramienta, «fines del Fondo», «temas» y «fracciones del art. 4 del Decreto» significan lo mismo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pasos de uso</t>
   </si>
   <si>
     <t xml:space="preserve">1. Parámetros: el Comité Técnico fija pesos, montos mínimo y máximo, umbrales y categorías antes de cada convocatoria.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. 1_Proyectos: registre cada propuesta (una fila por proyecto) con su fracción principal del art. 4 y hasta 3 fracciones secundarias.</t>
+    <t xml:space="preserve">2. 1_Proyectos: registre cada propuesta (una fila por proyecto) con su fracción principal (el fin del Fondo que atiende, según el art. 4 del Decreto) y hasta 3 fracciones secundarias.</t>
   </si>
   <si>
     <t xml:space="preserve">3. 2_Evaluación: en la misma fila, capture los 9 filtros (Sí/No) y, si el proyecto es elegible, las 14 calificaciones manuales (1 a 3). O4 y F5 se calculan solos.</t>
@@ -149,10 +155,10 @@
     <t xml:space="preserve">O2</t>
   </si>
   <si>
-    <t xml:space="preserve">Vinculación directa con un fin del art. 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿El objetivo general del proyecto atiende de forma directa al menos una fracción del art. 4?</t>
+    <t xml:space="preserve">Vinculación directa con un fin del Fondo (art. 4 del Decreto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿El objetivo general del proyecto atiende de forma directa al menos un fin del Fondo (una fracción del art. 4 del Decreto)?</t>
   </si>
   <si>
     <t xml:space="preserve">Sí: registra una fracción principal y su objetivo general la atiende de forma directa.</t>
@@ -329,10 +335,10 @@
     <t xml:space="preserve">Calificación (automática)</t>
   </si>
   <si>
-    <t xml:space="preserve">Contribución a varios fines del art. 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿A cuántas fracciones del art. 4 contribuye el proyecto?</t>
+    <t xml:space="preserve">Contribución a varios fines del Fondo (art. 4 del Decreto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿A cuántos fines del Fondo (fracciones del art. 4 del Decreto) contribuye el proyecto?</t>
   </si>
   <si>
     <t xml:space="preserve">3: contribuye a 3 o más fracciones.</t>
@@ -701,10 +707,10 @@
     <t xml:space="preserve">Art. 7 (integración multisectorial)</t>
   </si>
   <si>
-    <t xml:space="preserve">Temas financiables (art. 4 del Decreto) y criterios específicos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El requisito específico se verifica en el filtro O3; el indicador de impacto se usa en E1 y O5.</t>
+    <t xml:space="preserve">Temas financiables: los 16 fines del Fondo (art. 4 del Decreto) y sus criterios específicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El artículo 4 del Decreto por el que se constituye el Fideicomiso Público denominado Fondo Estatal Ambiental y Climático de Baja California Sur establece los fines del Fondo: 16 fracciones (I a XVI) que definen en qué puede invertir sus recursos. En esta herramienta, «fines del Fondo», «temas» y «fracciones del art. 4 del Decreto» significan lo mismo. El requisito específico se verifica en el filtro O3; el indicador de impacto se usa en E1 y O5.</t>
   </si>
   <si>
     <t xml:space="preserve">Fracción</t>
@@ -1022,7 +1028,7 @@
     <t xml:space="preserve">1. Registro de proyectos</t>
   </si>
   <si>
-    <t xml:space="preserve">Una fila por proyecto (filas 9 a 58). La fila de cada proyecto es la misma en 2_Evaluación.</t>
+    <t xml:space="preserve">Una fila por proyecto (filas 9 a 58). La fila de cada proyecto es la misma en 2_Evaluación. Las fracciones son los fines del Fondo del art. 4 del Decreto (hoja Temas).</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -2015,11 +2021,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="89229364"/>
-        <c:axId val="5677370"/>
+        <c:axId val="27787382"/>
+        <c:axId val="43246295"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="89229364"/>
+        <c:axId val="27787382"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2051,7 +2057,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5677370"/>
+        <c:crossAx val="43246295"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2059,7 +2065,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5677370"/>
+        <c:axId val="43246295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -2103,7 +2109,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89229364"/>
+        <c:crossAx val="27787382"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2346,7 +2352,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
@@ -2376,25 +2382,25 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-    </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2404,30 +2410,30 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-    </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2437,21 +2443,34 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="5" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2484,826 +2503,826 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G5" s="8"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G8" s="8"/>
       <c r="H8" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G9" s="8"/>
       <c r="H9" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G10" s="8"/>
       <c r="H10" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G11" s="8"/>
       <c r="H11" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J20" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J22" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J23" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J24" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J26" s="10" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J27" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J28" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J29" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3334,301 +3353,301 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3658,45 +3677,45 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>1</v>
@@ -3708,13 +3727,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D7" s="12" t="n">
         <v>2</v>
@@ -3726,13 +3745,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D8" s="12" t="n">
         <v>2</v>
@@ -3744,13 +3763,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>1</v>
@@ -3762,13 +3781,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D10" s="12" t="n">
         <v>1</v>
@@ -3780,13 +3799,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D11" s="12" t="n">
         <v>1</v>
@@ -3798,13 +3817,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D12" s="12" t="n">
         <v>1</v>
@@ -3816,13 +3835,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>1</v>
@@ -3834,13 +3853,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>1</v>
@@ -3852,13 +3871,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D15" s="12" t="n">
         <v>1</v>
@@ -3870,13 +3889,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D16" s="12" t="n">
         <v>1</v>
@@ -3888,13 +3907,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1</v>
@@ -3906,13 +3925,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>1</v>
@@ -3924,13 +3943,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>1</v>
@@ -3942,13 +3961,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>1</v>
@@ -3960,13 +3979,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>1</v>
@@ -3978,7 +3997,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="4" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D22" s="4" t="n">
         <f aca="false">SUM(D6:D21)</f>
@@ -3991,29 +4010,29 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C27" s="15" t="n">
         <f aca="false">COUNTIF($B$6:$B$21,A27)</f>
@@ -4026,7 +4045,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C28" s="15" t="n">
         <f aca="false">COUNTIF($B$6:$B$21,A28)</f>
@@ -4039,7 +4058,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C29" s="15" t="n">
         <f aca="false">COUNTIF($B$6:$B$21,A29)</f>
@@ -4052,7 +4071,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C30" s="15" t="n">
         <f aca="false">COUNTIF($B$6:$B$21,A30)</f>
@@ -4065,7 +4084,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C31" s="15" t="n">
         <f aca="false">COUNTIF($B$6:$B$21,A31)</f>
@@ -4078,34 +4097,34 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D37" s="17" t="n">
         <v>3</v>
@@ -4113,7 +4132,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D38" s="17" t="n">
         <v>2</v>
@@ -4121,7 +4140,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D39" s="18" t="n">
         <v>0.3</v>
@@ -4129,7 +4148,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D40" s="18" t="n">
         <v>0.1</v>
@@ -4137,7 +4156,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D41" s="17" t="n">
         <v>75</v>
@@ -4145,7 +4164,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D42" s="17" t="n">
         <v>50</v>
@@ -4153,42 +4172,42 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -4228,97 +4247,97 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I9" s="12"/>
       <c r="J9" s="15" t="str">
@@ -4340,40 +4359,40 @@
         <v>0.305555555555556</v>
       </c>
       <c r="O9" s="19" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="P9" s="19" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="R9" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="S9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
@@ -4396,37 +4415,37 @@
         <v>0.0909090909090909</v>
       </c>
       <c r="O10" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="P10" s="19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="R10" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="S10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
@@ -4453,31 +4472,31 @@
       <c r="P11" s="12"/>
       <c r="Q11" s="12"/>
       <c r="R11" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="S11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
@@ -4500,16 +4519,16 @@
         <v>0.4</v>
       </c>
       <c r="O12" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="P12" s="19" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="Q12" s="19" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="R12" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="S12" s="22"/>
     </row>
@@ -5938,22 +5957,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="M3" s="2" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D4" s="23" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E4" s="23"/>
       <c r="F4" s="23"/>
@@ -5964,7 +5983,7 @@
       <c r="K4" s="23"/>
       <c r="L4" s="23"/>
       <c r="M4" s="23" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="N4" s="23"/>
       <c r="O4" s="23"/>
@@ -5982,7 +6001,7 @@
       <c r="AA4" s="23"/>
       <c r="AB4" s="23"/>
       <c r="AC4" s="23" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="AD4" s="23"/>
       <c r="AE4" s="23"/>
@@ -6000,136 +6019,136 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="V5" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="X5" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="Y5" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="Z5" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="AA5" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="AB5" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="AC5" s="24" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="AD5" s="24" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="AE5" s="24" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="AF5" s="24" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="AG5" s="24" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="AH5" s="24" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="AI5" s="24" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="AJ5" s="24" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="AK5" s="24" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AL5" s="24" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AM5" s="24" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AN5" s="24" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AO5" s="24" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="AP5" s="24" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="AQ5" s="24" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="AR5" s="24" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6137,79 +6156,79 @@
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
       <c r="D6" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I6" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O6" s="25" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P6" s="25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="R6" s="25" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="S6" s="25" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="T6" s="25" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U6" s="25" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="V6" s="25" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="W6" s="25" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="X6" s="25" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="Y6" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="Z6" s="25" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AA6" s="25" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="AB6" s="25" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="AC6" s="24"/>
       <c r="AD6" s="24"/>
@@ -6233,79 +6252,79 @@
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
       <c r="D7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="H7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="J7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="N7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="O7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="P7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="Q7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="R7" s="25" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="S7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="T7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="U7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="V7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="W7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="X7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="Y7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="Z7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AB7" s="25" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AC7" s="24"/>
       <c r="AD7" s="24"/>
@@ -6329,31 +6348,31 @@
       <c r="B8" s="24"/>
       <c r="C8" s="24"/>
       <c r="D8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="M8" s="26" t="n">
         <f aca="false">Parámetros!$D$6</f>
@@ -6450,31 +6469,31 @@
         <v>IV</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M9" s="29" t="n">
         <f aca="false">IF(1_Proyectos!K9="","",IF(1_Proyectos!K9&gt;=Parámetros!$D$37,3,IF(1_Proyectos!K9&gt;=Parámetros!$D$38,2,1)))</f>
@@ -6579,7 +6598,7 @@
         <v/>
       </c>
       <c r="AP9" s="33" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AQ9" s="15" t="n">
         <f aca="false">IF(A9="","",IF(AL9&lt;&gt;"",AL9*1000000+N9*10000+O9*100+AI9-ROW()/1000,-ROW()))</f>
@@ -6604,31 +6623,31 @@
         <v>VI</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L10" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M10" s="29" t="n">
         <f aca="false">IF(1_Proyectos!K10="","",IF(1_Proyectos!K10&gt;=Parámetros!$D$37,3,IF(1_Proyectos!K10&gt;=Parámetros!$D$38,2,1)))</f>
@@ -6733,7 +6752,7 @@
         <v/>
       </c>
       <c r="AP10" s="33" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="AQ10" s="15" t="n">
         <f aca="false">IF(A10="","",IF(AL10&lt;&gt;"",AL10*1000000+N10*10000+O10*100+AI10-ROW()/1000,-ROW()))</f>
@@ -6758,31 +6777,31 @@
         <v>X</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="G11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K11" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L11" s="28" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="M11" s="29" t="n">
         <f aca="false">IF(1_Proyectos!K11="","",IF(1_Proyectos!K11&gt;=Parámetros!$D$37,3,IF(1_Proyectos!K11&gt;=Parámetros!$D$38,2,1)))</f>
@@ -6859,7 +6878,7 @@
         <v/>
       </c>
       <c r="AP11" s="33" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="AQ11" s="15" t="n">
         <f aca="false">IF(A11="","",IF(AL11&lt;&gt;"",AL11*1000000+N11*10000+O11*100+AI11-ROW()/1000,-ROW()))</f>
@@ -6884,29 +6903,29 @@
         <v>IX</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H12" s="34"/>
       <c r="I12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L12" s="28" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M12" s="29" t="n">
         <f aca="false">IF(1_Proyectos!K12="","",IF(1_Proyectos!K12&gt;=Parámetros!$D$37,3,IF(1_Proyectos!K12&gt;=Parámetros!$D$38,2,1)))</f>
@@ -6983,7 +7002,7 @@
         <v/>
       </c>
       <c r="AP12" s="33" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="AQ12" s="15" t="n">
         <f aca="false">IF(A12="","",IF(AL12&lt;&gt;"",AL12*1000000+N12*10000+O12*100+AI12-ROW()/1000,-ROW()))</f>
@@ -11960,22 +11979,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D5" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$A$9:$A$58,"?*")</f>
@@ -11984,7 +12003,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D6" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AD$9:$AD$58,"Elegible")</f>
@@ -11993,7 +12012,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D7" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AD$9:$AD$58,"No elegible")</f>
@@ -12002,7 +12021,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D8" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AD$9:$AD$58,"Pendiente")</f>
@@ -12011,7 +12030,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D9" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AM$9:$AM$58,"Alta")</f>
@@ -12020,7 +12039,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AM$9:$AM$58,"Media")</f>
@@ -12029,7 +12048,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D11" s="15" t="n">
         <f aca="false">COUNTIF(2_Evaluación!$AM$9:$AM$58,"Baja")</f>
@@ -12038,7 +12057,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D12" s="36" t="n">
         <f aca="false">SUMIF(2_Evaluación!$AD$9:$AD$58,"Elegible",1_Proyectos!$L$9:$L$58)</f>
@@ -12047,40 +12066,40 @@
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14579,18 +14598,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="E3" s="15" t="n">
         <f aca="false">IFERROR(MATCH(C3,1_Proyectos!$A$9:$A$58,0),"")</f>
@@ -14599,7 +14618,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C5" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$B$9:$B$58,$E$3)="","",INDEX(1_Proyectos!$B$9:$B$58,$E$3)))</f>
@@ -14611,7 +14630,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C6" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$C$9:$C$58,$E$3)="","",INDEX(1_Proyectos!$C$9:$C$58,$E$3)))</f>
@@ -14623,7 +14642,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C7" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$D$9:$D$58,$E$3)="","",INDEX(1_Proyectos!$D$9:$D$58,$E$3)))</f>
@@ -14635,7 +14654,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C8" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$E$9:$E$58,$E$3)="","",INDEX(1_Proyectos!$E$9:$E$58,$E$3)))</f>
@@ -14647,7 +14666,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C9" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$F$9:$F$58,$E$3)="","",INDEX(1_Proyectos!$F$9:$F$58,$E$3)))</f>
@@ -14659,7 +14678,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C10" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$J$9:$J$58,$E$3)="","",INDEX(1_Proyectos!$J$9:$J$58,$E$3)))</f>
@@ -14671,7 +14690,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C11" s="37" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$K$9:$K$58,$E$3)="","",INDEX(1_Proyectos!$K$9:$K$58,$E$3)))</f>
@@ -14683,7 +14702,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C12" s="38" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$L$9:$L$58,$E$3)="","",INDEX(1_Proyectos!$L$9:$L$58,$E$3)))</f>
@@ -14695,7 +14714,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C13" s="39" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$N$9:$N$58,$E$3)="","",INDEX(1_Proyectos!$N$9:$N$58,$E$3)))</f>
@@ -14707,7 +14726,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C14" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$O$9:$O$58,$E$3)="","",INDEX(1_Proyectos!$O$9:$O$58,$E$3)))</f>
@@ -14719,7 +14738,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C15" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$Q$9:$Q$58,$E$3)="","",INDEX(1_Proyectos!$Q$9:$Q$58,$E$3)))</f>
@@ -14731,7 +14750,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C16" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(1_Proyectos!$R$9:$R$58,$E$3)="","",INDEX(1_Proyectos!$R$9:$R$58,$E$3)))</f>
@@ -14743,33 +14762,33 @@
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="40" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D19" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$D$9:$D$58,$E$3)="","",INDEX(2_Evaluación!$D$9:$D$58,$E$3)))</f>
@@ -14783,13 +14802,13 @@
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="40" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D20" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$E$9:$E$58,$E$3)="","",INDEX(2_Evaluación!$E$9:$E$58,$E$3)))</f>
@@ -14803,13 +14822,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="40" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D21" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$F$9:$F$58,$E$3)="","",INDEX(2_Evaluación!$F$9:$F$58,$E$3)))</f>
@@ -14823,13 +14842,13 @@
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="40" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D22" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$G$9:$G$58,$E$3)="","",INDEX(2_Evaluación!$G$9:$G$58,$E$3)))</f>
@@ -14843,13 +14862,13 @@
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="40" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D23" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$H$9:$H$58,$E$3)="","",INDEX(2_Evaluación!$H$9:$H$58,$E$3)))</f>
@@ -14863,13 +14882,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="40" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D24" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$I$9:$I$58,$E$3)="","",INDEX(2_Evaluación!$I$9:$I$58,$E$3)))</f>
@@ -14883,13 +14902,13 @@
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="40" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D25" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$J$9:$J$58,$E$3)="","",INDEX(2_Evaluación!$J$9:$J$58,$E$3)))</f>
@@ -14903,13 +14922,13 @@
     </row>
     <row r="26" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="40" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D26" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$K$9:$K$58,$E$3)="","",INDEX(2_Evaluación!$K$9:$K$58,$E$3)))</f>
@@ -14923,13 +14942,13 @@
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D27" s="41" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$L$9:$L$58,$E$3)="","",INDEX(2_Evaluación!$L$9:$L$58,$E$3)))</f>
@@ -14943,13 +14962,13 @@
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="40" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D28" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$M$9:$M$58,$E$3)="","",INDEX(2_Evaluación!$M$9:$M$58,$E$3)))</f>
@@ -14963,13 +14982,13 @@
     </row>
     <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="40" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D29" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$N$9:$N$58,$E$3)="","",INDEX(2_Evaluación!$N$9:$N$58,$E$3)))</f>
@@ -14983,13 +15002,13 @@
     </row>
     <row r="30" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="40" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D30" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$O$9:$O$58,$E$3)="","",INDEX(2_Evaluación!$O$9:$O$58,$E$3)))</f>
@@ -15003,13 +15022,13 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="40" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D31" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$P$9:$P$58,$E$3)="","",INDEX(2_Evaluación!$P$9:$P$58,$E$3)))</f>
@@ -15023,13 +15042,13 @@
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="40" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D32" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$Q$9:$Q$58,$E$3)="","",INDEX(2_Evaluación!$Q$9:$Q$58,$E$3)))</f>
@@ -15043,13 +15062,13 @@
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D33" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$R$9:$R$58,$E$3)="","",INDEX(2_Evaluación!$R$9:$R$58,$E$3)))</f>
@@ -15063,13 +15082,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="40" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D34" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$S$9:$S$58,$E$3)="","",INDEX(2_Evaluación!$S$9:$S$58,$E$3)))</f>
@@ -15083,13 +15102,13 @@
     </row>
     <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D35" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$T$9:$T$58,$E$3)="","",INDEX(2_Evaluación!$T$9:$T$58,$E$3)))</f>
@@ -15103,13 +15122,13 @@
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="40" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D36" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$U$9:$U$58,$E$3)="","",INDEX(2_Evaluación!$U$9:$U$58,$E$3)))</f>
@@ -15123,13 +15142,13 @@
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="40" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D37" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$V$9:$V$58,$E$3)="","",INDEX(2_Evaluación!$V$9:$V$58,$E$3)))</f>
@@ -15143,13 +15162,13 @@
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D38" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$W$9:$W$58,$E$3)="","",INDEX(2_Evaluación!$W$9:$W$58,$E$3)))</f>
@@ -15163,13 +15182,13 @@
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="40" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D39" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$X$9:$X$58,$E$3)="","",INDEX(2_Evaluación!$X$9:$X$58,$E$3)))</f>
@@ -15183,13 +15202,13 @@
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="40" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D40" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$Y$9:$Y$58,$E$3)="","",INDEX(2_Evaluación!$Y$9:$Y$58,$E$3)))</f>
@@ -15203,13 +15222,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="40" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D41" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$Z$9:$Z$58,$E$3)="","",INDEX(2_Evaluación!$Z$9:$Z$58,$E$3)))</f>
@@ -15223,13 +15242,13 @@
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="40" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D42" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AA$9:$AA$58,$E$3)="","",INDEX(2_Evaluación!$AA$9:$AA$58,$E$3)))</f>
@@ -15243,13 +15262,13 @@
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="40" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D43" s="41" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AB$9:$AB$58,$E$3)="","",INDEX(2_Evaluación!$AB$9:$AB$58,$E$3)))</f>
@@ -15263,12 +15282,12 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C46" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AD$9:$AD$58,$E$3)="","",INDEX(2_Evaluación!$AD$9:$AD$58,$E$3)))</f>
@@ -15280,7 +15299,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C47" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AE$9:$AE$58,$E$3)="","",INDEX(2_Evaluación!$AE$9:$AE$58,$E$3)))</f>
@@ -15292,7 +15311,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C48" s="37" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AK$9:$AK$58,$E$3)="","",INDEX(2_Evaluación!$AK$9:$AK$58,$E$3)))</f>
@@ -15304,7 +15323,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C49" s="42" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AL$9:$AL$58,$E$3)="","",INDEX(2_Evaluación!$AL$9:$AL$58,$E$3)))</f>
@@ -15316,7 +15335,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C50" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AM$9:$AM$58,$E$3)="","",INDEX(2_Evaluación!$AM$9:$AM$58,$E$3)))</f>
@@ -15328,7 +15347,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C51" s="37" t="n">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AN$9:$AN$58,$E$3)="","",INDEX(2_Evaluación!$AN$9:$AN$58,$E$3)))</f>
@@ -15340,7 +15359,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C52" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AO$9:$AO$58,$E$3)="","",INDEX(2_Evaluación!$AO$9:$AO$58,$E$3)))</f>
@@ -15352,7 +15371,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C53" s="37" t="str">
         <f aca="false">IF($E$3="","",IF(INDEX(2_Evaluación!$AP$9:$AP$58,$E$3)="","",INDEX(2_Evaluación!$AP$9:$AP$58,$E$3)))</f>
@@ -15364,7 +15383,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>